<commit_message>
done paper review 1 of ACN
</commit_message>
<xml_diff>
--- a/Fall 2025/Advanced Computer Networks/Group presentation/Fall 2025/Fall 2025 Advanced Computer Networks (CEG-7450-01)_GradesExport_2025-08-30-14-54.xlsx
+++ b/Fall 2025/Advanced Computer Networks/Group presentation/Fall 2025/Fall 2025 Advanced Computer Networks (CEG-7450-01)_GradesExport_2025-08-30-14-54.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bwang\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhuwa\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{797138FE-1907-4B38-9B9C-43EFC4E3328F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="20115"/>
   </bookViews>
   <sheets>
     <sheet name="Grades" sheetId="1" r:id="rId1"/>
@@ -565,8 +564,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -702,7 +701,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -880,6 +879,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1043,11 +1048,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="16" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1422,11 +1429,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I40"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1440,7 +1447,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1460,7 +1467,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1480,7 +1487,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1500,7 +1507,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1520,7 +1527,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1540,7 +1547,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1560,7 +1567,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -1580,7 +1587,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1600,7 +1607,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -1620,7 +1627,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1640,7 +1647,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1660,7 +1667,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -1680,7 +1687,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>52</v>
       </c>
@@ -1700,7 +1707,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -1720,7 +1727,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>60</v>
       </c>
@@ -1740,7 +1747,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -1760,7 +1767,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>68</v>
       </c>
@@ -1780,7 +1787,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>72</v>
       </c>
@@ -1800,7 +1807,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -1820,7 +1827,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>80</v>
       </c>
@@ -1840,7 +1847,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>84</v>
       </c>
@@ -1860,7 +1867,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:9" s="2" customFormat="1">
       <c r="A23" s="2" t="s">
         <v>88</v>
       </c>
@@ -1880,7 +1887,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>92</v>
       </c>
@@ -1893,34 +1900,34 @@
       <c r="D24" t="s">
         <v>95</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24" s="5">
         <v>45954</v>
       </c>
       <c r="I24" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+    <row r="25" spans="1:9" s="4" customFormat="1">
+      <c r="A25" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25" s="5">
         <v>45954</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="4" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>100</v>
       </c>
@@ -1940,7 +1947,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -1960,7 +1967,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>108</v>
       </c>
@@ -1980,7 +1987,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>112</v>
       </c>
@@ -2000,7 +2007,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>116</v>
       </c>
@@ -2020,7 +2027,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>120</v>
       </c>
@@ -2040,7 +2047,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:9" s="2" customFormat="1">
       <c r="A32" s="2" t="s">
         <v>124</v>
       </c>
@@ -2060,7 +2067,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>128</v>
       </c>
@@ -2080,7 +2087,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>132</v>
       </c>
@@ -2100,7 +2107,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
         <v>136</v>
       </c>
@@ -2120,7 +2127,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>140</v>
       </c>
@@ -2140,7 +2147,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>144</v>
       </c>
@@ -2160,7 +2167,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>148</v>
       </c>
@@ -2180,7 +2187,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>152</v>
       </c>
@@ -2200,7 +2207,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>156</v>
       </c>

</xml_diff>